<commit_message>
Fix email UTF-8 (EmailMessage), update contacts: 318 rows, IT email + Core Banking email, rename dept
</commit_message>
<xml_diff>
--- a/it-helpdesk-bot/contacts.xlsx
+++ b/it-helpdesk-bot/contacts.xlsx
@@ -528,7 +528,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2178,7 +2178,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -3178,7 +3178,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -5428,7 +5428,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
@@ -7278,7 +7278,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -8278,7 +8278,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I158" t="inlineStr">
@@ -8378,7 +8378,7 @@
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
@@ -8528,7 +8528,7 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
@@ -8578,7 +8578,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
@@ -15778,7 +15778,7 @@
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
@@ -15828,7 +15828,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I308" t="inlineStr">
@@ -15878,7 +15878,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I309" t="inlineStr">
@@ -15928,7 +15928,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -16128,7 +16128,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>xuanbach6873932001@gmail.com</t>
+          <t>itservicedeskbank79@gmail.com</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -16278,7 +16278,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -16328,7 +16328,7 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>dung.pm@bank.com.vn</t>
+          <t>dungpm43@gmail.com</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">

</xml_diff>